<commit_message>
Update scraper docs and production baseline
</commit_message>
<xml_diff>
--- a/Ferguson Item Number Scraper Template.xlsx
+++ b/Ferguson Item Number Scraper Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://thehillgrp.sharepoint.com/sites/HMSSales/Shared Documents/Estimating Templates/Data/Automations/Ferguson PVF Item Number Scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_30D85E00F9810AF584FC99A0CED6A2EA156988F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD1A9165-D6E5-4E47-8C92-0443E63CFDC1}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_30D85E00F9810AF584FC99A0CED6A2EA156988F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{246A8D1E-5FE7-4DE8-A8CB-322B0D8251ED}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-33017" yWindow="-103" windowWidth="33120" windowHeight="18720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scraper Data" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
   <si>
     <t>Model</t>
   </si>
@@ -40,55 +40,166 @@
     <t>Cost</t>
   </si>
   <si>
-    <t>MN-ZMBBU0403</t>
+    <t>MN-ZMBLST4503</t>
   </si>
   <si>
-    <t>082647060883</t>
+    <t>082647063204</t>
   </si>
   <si>
-    <t>190838</t>
+    <t>1/2" BLK MALL 45 ST ELB</t>
   </si>
   <si>
-    <t>3/4" X 1/2" BLK MALL BUSHING</t>
+    <t>MN-ZMBLST4504</t>
   </si>
   <si>
-    <t>MN-ZMBBU0503</t>
+    <t>082647063211</t>
   </si>
   <si>
-    <t>082647060920</t>
+    <t>3/4" BLK MALL 45 ST ELB</t>
   </si>
   <si>
-    <t>190841</t>
+    <t>MN-ZMBLST4505</t>
   </si>
   <si>
-    <t>1" X 1/2" BLK MALL BUSHING</t>
+    <t>082647063228</t>
   </si>
   <si>
-    <t>MN-ZMBBU0504</t>
+    <t>1" BLK MALL 45 ST ELB</t>
   </si>
   <si>
-    <t>082647060937</t>
+    <t>MN-ZMBLST4506</t>
   </si>
   <si>
-    <t>190842</t>
+    <t>082647063235</t>
   </si>
   <si>
-    <t>1" X 3/4" BLK MALL BUSHING</t>
+    <t>1-1/4" BLK MALL 45 ST ELB</t>
   </si>
   <si>
-    <t>MN-ZMBBU0603</t>
+    <t>MN-ZMBLST4507</t>
   </si>
   <si>
-    <t>082647060975</t>
+    <t>082647063242</t>
   </si>
   <si>
-    <t>190843</t>
+    <t>1-1/2" BLK MALL 45 ST ELB</t>
   </si>
   <si>
-    <t>1-1/4" X 1/2" BLK MALL BUSHING</t>
+    <t>MN-ZMBLST4508</t>
   </si>
   <si>
-    <t>GALVANIZED</t>
+    <t>082647063259</t>
+  </si>
+  <si>
+    <t>2" BLK MALL 45 ST ELB</t>
+  </si>
+  <si>
+    <t>MN-ZMBLST4509</t>
+  </si>
+  <si>
+    <t>082647063266</t>
+  </si>
+  <si>
+    <t>2-1/2" BLK MALL 45 ST ELB</t>
+  </si>
+  <si>
+    <t>MN-ZMBLST4510</t>
+  </si>
+  <si>
+    <t>082647063273</t>
+  </si>
+  <si>
+    <t>3" BLK MALL 45 ST ELB</t>
+  </si>
+  <si>
+    <t>MN-ZMBLST4511</t>
+  </si>
+  <si>
+    <t>082647133778</t>
+  </si>
+  <si>
+    <t>4" BLK MALL 45 ST ELB</t>
+  </si>
+  <si>
+    <t>MN-ZMBLST9003</t>
+  </si>
+  <si>
+    <t>082647063327</t>
+  </si>
+  <si>
+    <t>1/2" BLK MALL 90 ST ELB</t>
+  </si>
+  <si>
+    <t>MN-ZMBLST9004</t>
+  </si>
+  <si>
+    <t>082647063334</t>
+  </si>
+  <si>
+    <t>3/4" BLK MALL 90 ST ELB</t>
+  </si>
+  <si>
+    <t>MN-ZMBLST9005</t>
+  </si>
+  <si>
+    <t>082647063341</t>
+  </si>
+  <si>
+    <t>1" BLK MALL 90 ST ELB</t>
+  </si>
+  <si>
+    <t>MN-ZMBLST9006</t>
+  </si>
+  <si>
+    <t>082647063358</t>
+  </si>
+  <si>
+    <t>1-1/4" BLK MALL 90 ST ELB</t>
+  </si>
+  <si>
+    <t>MN-ZMBLST9007</t>
+  </si>
+  <si>
+    <t>082647063365</t>
+  </si>
+  <si>
+    <t>1-1/2" BLK MALL 90 ST ELB</t>
+  </si>
+  <si>
+    <t>MN-ZMBLST9008</t>
+  </si>
+  <si>
+    <t>082647063372</t>
+  </si>
+  <si>
+    <t>2" BLK MALL 90 ST ELB</t>
+  </si>
+  <si>
+    <t>MN-ZMBLST9009</t>
+  </si>
+  <si>
+    <t>082647063389</t>
+  </si>
+  <si>
+    <t>2-1/2" BLK MALL 90 ST ELB</t>
+  </si>
+  <si>
+    <t>MN-ZMBLST9010</t>
+  </si>
+  <si>
+    <t>082647063396</t>
+  </si>
+  <si>
+    <t>3" BLK MALL 90 ST ELB</t>
+  </si>
+  <si>
+    <t>MN-ZMBLST9011</t>
+  </si>
+  <si>
+    <t>082647063402</t>
+  </si>
+  <si>
+    <t>4" BLK MALL 90 ST ELB</t>
   </si>
 </sst>
 </file>
@@ -143,7 +254,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -153,12 +264,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="1"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -193,7 +298,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -213,10 +318,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -226,6 +327,9 @@
     <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -524,19 +628,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18.899999999999999" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
     </row>
@@ -547,163 +651,231 @@
       <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="1"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="1">
-        <v>3.97</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A3" s="3" t="s">
+      <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3"/>
+      <c r="D3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="E3" s="1"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="1">
-        <v>4.09</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A4" s="3" t="s">
+      <c r="C4" s="3"/>
+      <c r="D4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="C5" s="3"/>
+      <c r="D5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="1">
-        <v>4.09</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A5" s="3" t="s">
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C6" s="3"/>
+      <c r="D6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="1">
-        <v>5.86</v>
+      <c r="B7" s="3" t="s">
+        <v>21</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
       <c r="C7" s="3"/>
-      <c r="D7" s="5"/>
+      <c r="D7" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="E7" s="1"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
+      <c r="A8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="C8" s="3"/>
-      <c r="D8" s="5"/>
+      <c r="D8" s="5" t="s">
+        <v>25</v>
+      </c>
       <c r="E8" s="1"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
+      <c r="A9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>27</v>
+      </c>
       <c r="C9" s="3"/>
-      <c r="D9" s="5"/>
+      <c r="D9" s="5" t="s">
+        <v>28</v>
+      </c>
       <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
+      <c r="A10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>30</v>
+      </c>
       <c r="C10" s="3"/>
-      <c r="D10" s="5"/>
+      <c r="D10" s="5" t="s">
+        <v>31</v>
+      </c>
       <c r="E10" s="1"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
+      <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>33</v>
+      </c>
       <c r="C11" s="3"/>
-      <c r="D11" s="5"/>
+      <c r="D11" s="5" t="s">
+        <v>34</v>
+      </c>
       <c r="E11" s="1"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
+      <c r="A12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>36</v>
+      </c>
       <c r="C12" s="3"/>
-      <c r="D12" s="5"/>
+      <c r="D12" s="5" t="s">
+        <v>37</v>
+      </c>
       <c r="E12" s="1"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
+      <c r="A13" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>39</v>
+      </c>
       <c r="C13" s="3"/>
-      <c r="D13" s="5"/>
+      <c r="D13" s="5" t="s">
+        <v>40</v>
+      </c>
       <c r="E13" s="1"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
+      <c r="A14" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>42</v>
+      </c>
       <c r="C14" s="3"/>
-      <c r="D14" s="5"/>
+      <c r="D14" s="5" t="s">
+        <v>43</v>
+      </c>
       <c r="E14" s="1"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
+      <c r="A15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>45</v>
+      </c>
       <c r="C15" s="3"/>
-      <c r="D15" s="5"/>
+      <c r="D15" s="5" t="s">
+        <v>46</v>
+      </c>
       <c r="E15" s="1"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
+      <c r="A16" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>48</v>
+      </c>
       <c r="C16" s="3"/>
-      <c r="D16" s="5"/>
+      <c r="D16" s="5" t="s">
+        <v>49</v>
+      </c>
       <c r="E16" s="1"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
+      <c r="A17" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>51</v>
+      </c>
       <c r="C17" s="3"/>
-      <c r="D17" s="5"/>
+      <c r="D17" s="5" t="s">
+        <v>52</v>
+      </c>
       <c r="E17" s="1"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
+      <c r="A18" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>54</v>
+      </c>
       <c r="C18" s="3"/>
-      <c r="D18" s="5"/>
+      <c r="D18" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="E18" s="1"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
+      <c r="A19" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>57</v>
+      </c>
       <c r="C19" s="3"/>
-      <c r="D19" s="5"/>
+      <c r="D19" s="5" t="s">
+        <v>58</v>
+      </c>
       <c r="E19" s="1"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.4">
@@ -2210,11 +2382,9 @@
       <c r="C234" s="3"/>
       <c r="D234" s="5"/>
       <c r="E234" s="1"/>
-      <c r="F234" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G234" s="8"/>
-      <c r="H234" s="8"/>
+      <c r="F234" s="11"/>
+      <c r="G234" s="12"/>
+      <c r="H234" s="10"/>
     </row>
     <row r="235" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A235" s="3"/>
@@ -6844,9 +7014,6 @@
       <c r="E895" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="F234:H234"/>
-  </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.2" right="0.2" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="55" fitToHeight="2000" orientation="landscape"/>
@@ -6857,17 +7024,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2276e458-9330-43ee-9396-75b7556b0046">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="0ac4a9bb-a261-4909-a4e8-84f9b1bc6880" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -6876,7 +7032,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003F467A083698CA4789F0594320E4680B" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="24b28c0f665927f5b40f55c356d4c1ec">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2276e458-9330-43ee-9396-75b7556b0046" xmlns:ns3="0ac4a9bb-a261-4909-a4e8-84f9b1bc6880" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2f3bba30793de4cdc486a18f07324894" ns2:_="" ns3:_="">
     <xsd:import namespace="2276e458-9330-43ee-9396-75b7556b0046"/>
@@ -7071,18 +7227,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6EB27CD9-3366-42F1-BEB9-40993F77F1BD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="2276e458-9330-43ee-9396-75b7556b0046"/>
-    <ds:schemaRef ds:uri="0ac4a9bb-a261-4909-a4e8-84f9b1bc6880"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2276e458-9330-43ee-9396-75b7556b0046">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="0ac4a9bb-a261-4909-a4e8-84f9b1bc6880" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82C331F8-1602-4D34-B284-51B7D3959812}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -7090,7 +7246,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A64D3079-3FC0-4701-B67F-6338C6C0CFA2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7107,4 +7263,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6EB27CD9-3366-42F1-BEB9-40993F77F1BD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2276e458-9330-43ee-9396-75b7556b0046"/>
+    <ds:schemaRef ds:uri="0ac4a9bb-a261-4909-a4e8-84f9b1bc6880"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>